<commit_message>
Bug fixing on Crossover
</commit_message>
<xml_diff>
--- a/evaluation_results/Charts_and Tables.xlsx
+++ b/evaluation_results/Charts_and Tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sethm\Final Year Project\Retail-Stock-Analytics-Dashboard\evaluation_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4C24DC1C-FFF6-4884-A35E-7B74C4B92F75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F64C4231-AB42-44C4-B4DB-F0221572EA21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{11AB1E82-AA25-430D-9850-B42BE7948BE5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{11AB1E82-AA25-430D-9850-B42BE7948BE5}"/>
   </bookViews>
   <sheets>
     <sheet name="Table 1" sheetId="10" r:id="rId1"/>
@@ -19,22 +19,22 @@
     <sheet name="Table 4" sheetId="13" r:id="rId4"/>
     <sheet name="Sheet14" sheetId="14" r:id="rId5"/>
     <sheet name="Sheet15" sheetId="15" r:id="rId6"/>
-    <sheet name="Accuracy - &gt;" sheetId="9" r:id="rId7"/>
-    <sheet name="signals" sheetId="5" r:id="rId8"/>
-    <sheet name="summary" sheetId="4" r:id="rId9"/>
-    <sheet name="kadia" sheetId="3" r:id="rId10"/>
-    <sheet name="agreement_matrix" sheetId="2" r:id="rId11"/>
-    <sheet name="Sheet6" sheetId="6" r:id="rId12"/>
-    <sheet name="Accuracy" sheetId="7" r:id="rId13"/>
-    <sheet name="Sharpe" sheetId="8" r:id="rId14"/>
+    <sheet name="Sheet1" sheetId="16" r:id="rId7"/>
+    <sheet name="Accuracy - &gt;" sheetId="9" r:id="rId8"/>
+    <sheet name="signals" sheetId="5" r:id="rId9"/>
+    <sheet name="summary" sheetId="4" r:id="rId10"/>
+    <sheet name="kadia" sheetId="3" r:id="rId11"/>
+    <sheet name="agreement_matrix" sheetId="2" r:id="rId12"/>
+    <sheet name="Sheet6" sheetId="6" r:id="rId13"/>
+    <sheet name="Accuracy" sheetId="7" r:id="rId14"/>
+    <sheet name="Sharpe" sheetId="8" r:id="rId15"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId15"/>
     <externalReference r:id="rId16"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="17" r:id="rId17"/>
+    <pivotCache cacheId="0" r:id="rId17"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="255">
   <si>
     <t>rule\rl</t>
   </si>
@@ -1118,13 +1118,57 @@
   <si>
     <t>General-purpose dictionaries mislabel 75% of finance-specific negatives</t>
   </si>
+  <si>
+    <t>CHTR</t>
+  </si>
+  <si>
+    <t>CMCSA</t>
+  </si>
+  <si>
+    <t>DIS</t>
+  </si>
+  <si>
+    <t>EA</t>
+  </si>
+  <si>
+    <t>FOX</t>
+  </si>
+  <si>
+    <t>FOXA</t>
+  </si>
+  <si>
+    <t>GOOG</t>
+  </si>
+  <si>
+    <t>LYV</t>
+  </si>
+  <si>
+    <t>PEER_MEDIAN</t>
+  </si>
+  <si>
+    <t>P/E Ratio</t>
+  </si>
+  <si>
+    <t>ROE</t>
+  </si>
+  <si>
+    <t>Net Margin</t>
+  </si>
+  <si>
+    <t>Revenue Growth</t>
+  </si>
+  <si>
+    <t>Debt/Equity</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="3">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="22" x14ac:knownFonts="1">
     <font>
@@ -1235,20 +1279,20 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF1F3864"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF1F3864"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1580,12 +1624,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
@@ -1608,42 +1653,23 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1688,7 +1714,6 @@
     <xf numFmtId="2" fontId="17" fillId="8" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
@@ -1701,19 +1726,7 @@
     <xf numFmtId="0" fontId="13" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1728,12 +1741,6 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
@@ -1742,15 +1749,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1798,8 +1796,72 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="15" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="13" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
+    <cellStyle name="Comma" xfId="3" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{6F6C185B-43B3-47DA-93A2-531AA1D94C20}"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
@@ -6343,99 +6405,6 @@
       <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
-      <sheetName val="Overview"/>
-      <sheetName val="Raw_Signals"/>
-      <sheetName val="Raw_Agreement"/>
-      <sheetName val="Raw_Kadia"/>
-      <sheetName val="Table_7.1_Agreement"/>
-      <sheetName val="Table_7.2_Markout"/>
-      <sheetName val="Table_7.3_Kadia"/>
-      <sheetName val="Fig_7.1_Agreement"/>
-      <sheetName val="Fig_7.2_Horizon"/>
-      <sheetName val="Fig_7.3_Accuracy"/>
-      <sheetName val="Fig_7.4_Sharpe"/>
-      <sheetName val="Fig_7.5_Scatter"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8">
-        <row r="4">
-          <cell r="B4" t="str">
-            <v>Avg Markout (%)</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5">
-            <v>1</v>
-          </cell>
-          <cell r="B5">
-            <v>2.3154727272727276</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6">
-            <v>2</v>
-          </cell>
-          <cell r="B6">
-            <v>1.8436363636363637</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7">
-            <v>3</v>
-          </cell>
-          <cell r="B7">
-            <v>2.6672818181818179</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8">
-            <v>5</v>
-          </cell>
-          <cell r="B8">
-            <v>2.4910318181818183</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9">
-            <v>10</v>
-          </cell>
-          <cell r="B9">
-            <v>4.9059727272727267</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10">
-            <v>21</v>
-          </cell>
-          <cell r="B10">
-            <v>5.9269045454545468</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-      <xxl21:relativeUrl r:id="rId3"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
       <sheetName val="Raw_Data"/>
       <sheetName val="Fig_7.3_Accuracy"/>
       <sheetName val="Fig_7.4_Sharpe"/>
@@ -6689,216 +6658,12 @@
           <cell r="B4" t="str">
             <v>Accuracy (%)</v>
           </cell>
-          <cell r="C4" t="str">
-            <v>Kadia benchmark (%)</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5" t="str">
-            <v>GOOGL</v>
-          </cell>
-          <cell r="B5">
-            <v>100</v>
-          </cell>
-          <cell r="C5">
-            <v>85</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6" t="str">
-            <v>APP</v>
-          </cell>
-          <cell r="B6">
-            <v>81.25</v>
-          </cell>
-          <cell r="C6">
-            <v>85</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7" t="str">
-            <v>JPM</v>
-          </cell>
-          <cell r="B7">
-            <v>75</v>
-          </cell>
-          <cell r="C7">
-            <v>85</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8" t="str">
-            <v>DASH</v>
-          </cell>
-          <cell r="B8">
-            <v>71.430000000000007</v>
-          </cell>
-          <cell r="C8">
-            <v>85</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9" t="str">
-            <v>CVNA</v>
-          </cell>
-          <cell r="B9">
-            <v>66.67</v>
-          </cell>
-          <cell r="C9">
-            <v>85</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10" t="str">
-            <v>AAPL</v>
-          </cell>
-          <cell r="B10">
-            <v>66.67</v>
-          </cell>
-          <cell r="C10">
-            <v>85</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11" t="str">
-            <v>ISRG</v>
-          </cell>
-          <cell r="B11">
-            <v>33.33</v>
-          </cell>
-          <cell r="C11">
-            <v>85</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="A12" t="str">
-            <v>BAX</v>
-          </cell>
-          <cell r="B12">
-            <v>0</v>
-          </cell>
-          <cell r="C12">
-            <v>85</v>
-          </cell>
         </row>
       </sheetData>
       <sheetData sheetId="2">
         <row r="4">
           <cell r="B4" t="str">
             <v>Sharpe (annualised)</v>
-          </cell>
-          <cell r="C4" t="str">
-            <v>Kadia benchmark</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5" t="str">
-            <v>APP</v>
-          </cell>
-          <cell r="B5">
-            <v>2.09</v>
-          </cell>
-          <cell r="C5">
-            <v>2.27</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6" t="str">
-            <v>DASH</v>
-          </cell>
-          <cell r="B6">
-            <v>1.57</v>
-          </cell>
-          <cell r="C6">
-            <v>2.27</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7" t="str">
-            <v>GOOGL</v>
-          </cell>
-          <cell r="B7">
-            <v>1.54</v>
-          </cell>
-          <cell r="C7">
-            <v>2.27</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8" t="str">
-            <v>CVNA</v>
-          </cell>
-          <cell r="B8">
-            <v>1.44</v>
-          </cell>
-          <cell r="C8">
-            <v>2.27</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9" t="str">
-            <v>JPM</v>
-          </cell>
-          <cell r="B9">
-            <v>1.19</v>
-          </cell>
-          <cell r="C9">
-            <v>2.27</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10" t="str">
-            <v>AMZN</v>
-          </cell>
-          <cell r="B10">
-            <v>1.18</v>
-          </cell>
-          <cell r="C10">
-            <v>2.27</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11" t="str">
-            <v>AAPL</v>
-          </cell>
-          <cell r="B11">
-            <v>1.02</v>
-          </cell>
-          <cell r="C11">
-            <v>2.27</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="A12" t="str">
-            <v>TSLA</v>
-          </cell>
-          <cell r="B12">
-            <v>0.91</v>
-          </cell>
-          <cell r="C12">
-            <v>2.27</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="A13" t="str">
-            <v>ISRG</v>
-          </cell>
-          <cell r="B13">
-            <v>0.66</v>
-          </cell>
-          <cell r="C13">
-            <v>2.27</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14" t="str">
-            <v>BAX</v>
-          </cell>
-          <cell r="B14">
-            <v>-0.71</v>
-          </cell>
-          <cell r="C14">
-            <v>2.27</v>
           </cell>
         </row>
       </sheetData>
@@ -7191,7 +6956,169 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A83298BD-D10D-42D6-913D-7F64ACE9C0A4}" name="PivotTable4" cacheId="17" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6C0EFD4B-4A2A-445E-9C86-D742E9BEAD5D}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A16:F17" firstHeaderRow="0" firstDataRow="1" firstDataCol="0" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="14">
+    <pivotField axis="axisPage" showAll="0">
+      <items count="10">
+        <item x="8"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowItems count="1">
+    <i/>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+    <i i="2">
+      <x v="2"/>
+    </i>
+    <i i="3">
+      <x v="3"/>
+    </i>
+    <i i="4">
+      <x v="4"/>
+    </i>
+    <i i="5">
+      <x v="5"/>
+    </i>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="0" item="0" hier="-1"/>
+  </pageFields>
+  <dataFields count="6">
+    <dataField name="Sum of win_rate_1d" fld="3" baseField="0" baseItem="0"/>
+    <dataField name="Sum of win_rate_2d" fld="5" baseField="0" baseItem="0"/>
+    <dataField name="Sum of win_rate_3d" fld="7" baseField="0" baseItem="0"/>
+    <dataField name="Sum of win_rate_5d" fld="9" baseField="0" baseItem="0"/>
+    <dataField name="Sum of win_rate_10d" fld="11" baseField="0" baseItem="0"/>
+    <dataField name="Sum of win_rate_21d" fld="13" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D4792ADA-5F79-45FE-A234-E21D0578C084}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A11:F12" firstHeaderRow="0" firstDataRow="1" firstDataCol="0" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="14">
+    <pivotField axis="axisPage" showAll="0">
+      <items count="10">
+        <item x="8"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowItems count="1">
+    <i/>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+    <i i="2">
+      <x v="2"/>
+    </i>
+    <i i="3">
+      <x v="3"/>
+    </i>
+    <i i="4">
+      <x v="4"/>
+    </i>
+    <i i="5">
+      <x v="5"/>
+    </i>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="0" item="0" hier="-1"/>
+  </pageFields>
+  <dataFields count="6">
+    <dataField name="Sum of avg_markout_1d" fld="2" baseField="0" baseItem="0"/>
+    <dataField name="Sum of avg_markout_2d" fld="4" baseField="0" baseItem="0"/>
+    <dataField name="Sum of avg_markout_3d" fld="6" baseField="0" baseItem="0"/>
+    <dataField name="Sum of avg_markout_5d" fld="8" baseField="0" baseItem="0"/>
+    <dataField name="Sum of avg_markout_10d" fld="10" baseField="0" baseItem="0"/>
+    <dataField name="Sum of avg_markout_21d" fld="12" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A83298BD-D10D-42D6-913D-7F64ACE9C0A4}" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A43:G52" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
@@ -7279,168 +7206,6 @@
   </colItems>
   <dataFields count="6">
     <dataField name="Average of avg_markout_1d" fld="2" subtotal="average" baseField="0" baseItem="0"/>
-    <dataField name="Sum of avg_markout_2d" fld="4" baseField="0" baseItem="0"/>
-    <dataField name="Sum of avg_markout_3d" fld="6" baseField="0" baseItem="0"/>
-    <dataField name="Sum of avg_markout_5d" fld="8" baseField="0" baseItem="0"/>
-    <dataField name="Sum of avg_markout_10d" fld="10" baseField="0" baseItem="0"/>
-    <dataField name="Sum of avg_markout_21d" fld="12" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6C0EFD4B-4A2A-445E-9C86-D742E9BEAD5D}" name="PivotTable3" cacheId="17" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A16:F17" firstHeaderRow="0" firstDataRow="1" firstDataCol="0" rowPageCount="1" colPageCount="1"/>
-  <pivotFields count="14">
-    <pivotField axis="axisPage" showAll="0">
-      <items count="10">
-        <item x="8"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-  </pivotFields>
-  <rowItems count="1">
-    <i/>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="6">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-    <i i="2">
-      <x v="2"/>
-    </i>
-    <i i="3">
-      <x v="3"/>
-    </i>
-    <i i="4">
-      <x v="4"/>
-    </i>
-    <i i="5">
-      <x v="5"/>
-    </i>
-  </colItems>
-  <pageFields count="1">
-    <pageField fld="0" item="0" hier="-1"/>
-  </pageFields>
-  <dataFields count="6">
-    <dataField name="Sum of win_rate_1d" fld="3" baseField="0" baseItem="0"/>
-    <dataField name="Sum of win_rate_2d" fld="5" baseField="0" baseItem="0"/>
-    <dataField name="Sum of win_rate_3d" fld="7" baseField="0" baseItem="0"/>
-    <dataField name="Sum of win_rate_5d" fld="9" baseField="0" baseItem="0"/>
-    <dataField name="Sum of win_rate_10d" fld="11" baseField="0" baseItem="0"/>
-    <dataField name="Sum of win_rate_21d" fld="13" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D4792ADA-5F79-45FE-A234-E21D0578C084}" name="PivotTable2" cacheId="17" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A11:F12" firstHeaderRow="0" firstDataRow="1" firstDataCol="0" rowPageCount="1" colPageCount="1"/>
-  <pivotFields count="14">
-    <pivotField axis="axisPage" showAll="0">
-      <items count="10">
-        <item x="8"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowItems count="1">
-    <i/>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="6">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-    <i i="2">
-      <x v="2"/>
-    </i>
-    <i i="3">
-      <x v="3"/>
-    </i>
-    <i i="4">
-      <x v="4"/>
-    </i>
-    <i i="5">
-      <x v="5"/>
-    </i>
-  </colItems>
-  <pageFields count="1">
-    <pageField fld="0" item="0" hier="-1"/>
-  </pageFields>
-  <dataFields count="6">
-    <dataField name="Sum of avg_markout_1d" fld="2" baseField="0" baseItem="0"/>
     <dataField name="Sum of avg_markout_2d" fld="4" baseField="0" baseItem="0"/>
     <dataField name="Sum of avg_markout_3d" fld="6" baseField="0" baseItem="0"/>
     <dataField name="Sum of avg_markout_5d" fld="8" baseField="0" baseItem="0"/>
@@ -7780,128 +7545,128 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" style="38" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="59" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="44" t="s">
         <v>81</v>
       </c>
-      <c r="B1" s="62" t="s">
+      <c r="B1" s="45" t="s">
         <v>82</v>
       </c>
-      <c r="C1" s="61" t="s">
+      <c r="C1" s="44" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="31" t="s">
         <v>222</v>
       </c>
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="41" t="s">
         <v>84</v>
       </c>
-      <c r="C2" s="39" t="s">
+      <c r="C2" s="31" t="s">
         <v>223</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="32" t="s">
         <v>224</v>
       </c>
-      <c r="B3" s="55" t="s">
+      <c r="B3" s="41" t="s">
         <v>84</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="32" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="39" t="s">
+      <c r="A4" s="31" t="s">
         <v>225</v>
       </c>
-      <c r="B4" s="55" t="s">
+      <c r="B4" s="41" t="s">
         <v>84</v>
       </c>
-      <c r="C4" s="39" t="s">
+      <c r="C4" s="31" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="39" t="s">
+      <c r="A5" s="31" t="s">
         <v>227</v>
       </c>
-      <c r="B5" s="55" t="s">
+      <c r="B5" s="41" t="s">
         <v>86</v>
       </c>
-      <c r="C5" s="39" t="s">
+      <c r="C5" s="31" t="s">
         <v>228</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="39" t="s">
+      <c r="A6" s="31" t="s">
         <v>229</v>
       </c>
-      <c r="B6" s="55" t="s">
+      <c r="B6" s="41" t="s">
         <v>87</v>
       </c>
-      <c r="C6" s="39" t="s">
+      <c r="C6" s="31" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="39" t="s">
+      <c r="A7" s="31" t="s">
         <v>230</v>
       </c>
-      <c r="B7" s="55" t="s">
+      <c r="B7" s="41" t="s">
         <v>87</v>
       </c>
-      <c r="C7" s="39" t="s">
+      <c r="C7" s="31" t="s">
         <v>231</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="39" t="s">
+      <c r="A8" s="31" t="s">
         <v>232</v>
       </c>
-      <c r="B8" s="55" t="s">
+      <c r="B8" s="41" t="s">
         <v>87</v>
       </c>
-      <c r="C8" s="39" t="s">
+      <c r="C8" s="31" t="s">
         <v>233</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="39" t="s">
+      <c r="A9" s="31" t="s">
         <v>234</v>
       </c>
-      <c r="B9" s="55" t="s">
+      <c r="B9" s="41" t="s">
         <v>88</v>
       </c>
-      <c r="C9" s="39" t="s">
+      <c r="C9" s="31" t="s">
         <v>240</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="39" t="s">
+      <c r="A10" s="31" t="s">
         <v>235</v>
       </c>
-      <c r="B10" s="55" t="s">
+      <c r="B10" s="41" t="s">
         <v>88</v>
       </c>
-      <c r="C10" s="39" t="s">
+      <c r="C10" s="31" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="39" t="s">
+      <c r="A11" s="31" t="s">
         <v>237</v>
       </c>
-      <c r="B11" s="55" t="s">
+      <c r="B11" s="41" t="s">
         <v>89</v>
       </c>
-      <c r="C11" s="39" t="s">
+      <c r="C11" s="31" t="s">
         <v>239</v>
       </c>
     </row>
@@ -7911,6 +7676,456 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{997BFE89-0423-4747-91F1-EB3B75F2F832}">
+  <dimension ref="A1:N10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I1" t="s">
+        <v>29</v>
+      </c>
+      <c r="J1" t="s">
+        <v>30</v>
+      </c>
+      <c r="K1" t="s">
+        <v>31</v>
+      </c>
+      <c r="L1" t="s">
+        <v>32</v>
+      </c>
+      <c r="M1" t="s">
+        <v>33</v>
+      </c>
+      <c r="N1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2">
+        <v>3</v>
+      </c>
+      <c r="C2">
+        <v>1.1539999999999999</v>
+      </c>
+      <c r="D2">
+        <v>100</v>
+      </c>
+      <c r="E2">
+        <v>1.226</v>
+      </c>
+      <c r="F2">
+        <v>100</v>
+      </c>
+      <c r="G2">
+        <v>9.0999999999999998E-2</v>
+      </c>
+      <c r="H2">
+        <v>66.67</v>
+      </c>
+      <c r="I2">
+        <v>-0.247</v>
+      </c>
+      <c r="J2">
+        <v>33.33</v>
+      </c>
+      <c r="K2">
+        <v>-1.7989999999999999</v>
+      </c>
+      <c r="L2">
+        <v>66.67</v>
+      </c>
+      <c r="M2">
+        <v>-6.0869999999999997</v>
+      </c>
+      <c r="N2">
+        <v>33.33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3">
+        <v>4</v>
+      </c>
+      <c r="C3">
+        <v>-0.57999999999999996</v>
+      </c>
+      <c r="D3">
+        <v>25</v>
+      </c>
+      <c r="E3">
+        <v>0.13300000000000001</v>
+      </c>
+      <c r="F3">
+        <v>25</v>
+      </c>
+      <c r="G3">
+        <v>-0.64500000000000002</v>
+      </c>
+      <c r="H3">
+        <v>25</v>
+      </c>
+      <c r="I3">
+        <v>-0.53900000000000003</v>
+      </c>
+      <c r="J3">
+        <v>25</v>
+      </c>
+      <c r="K3">
+        <v>1.611</v>
+      </c>
+      <c r="L3">
+        <v>25</v>
+      </c>
+      <c r="M3">
+        <v>15.06</v>
+      </c>
+      <c r="N3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <v>-1.1359999999999999</v>
+      </c>
+      <c r="D4">
+        <v>33.33</v>
+      </c>
+      <c r="E4">
+        <v>-1.0109999999999999</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>-0.86299999999999999</v>
+      </c>
+      <c r="H4">
+        <v>33.33</v>
+      </c>
+      <c r="I4">
+        <v>-0.21299999999999999</v>
+      </c>
+      <c r="J4">
+        <v>66.67</v>
+      </c>
+      <c r="K4">
+        <v>2.76</v>
+      </c>
+      <c r="L4">
+        <v>66.67</v>
+      </c>
+      <c r="M4">
+        <v>7.1580000000000004</v>
+      </c>
+      <c r="N4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>32.093000000000004</v>
+      </c>
+      <c r="D5">
+        <v>100</v>
+      </c>
+      <c r="E5">
+        <v>33.332999999999998</v>
+      </c>
+      <c r="F5">
+        <v>100</v>
+      </c>
+      <c r="G5">
+        <v>53.444000000000003</v>
+      </c>
+      <c r="H5">
+        <v>100</v>
+      </c>
+      <c r="I5">
+        <v>44.877000000000002</v>
+      </c>
+      <c r="J5">
+        <v>100</v>
+      </c>
+      <c r="K5">
+        <v>51.631</v>
+      </c>
+      <c r="L5">
+        <v>100</v>
+      </c>
+      <c r="M5">
+        <v>63.975999999999999</v>
+      </c>
+      <c r="N5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>5.3710000000000004</v>
+      </c>
+      <c r="D6">
+        <v>100</v>
+      </c>
+      <c r="E6">
+        <v>3.0259999999999998</v>
+      </c>
+      <c r="F6">
+        <v>100</v>
+      </c>
+      <c r="G6">
+        <v>5.2670000000000003</v>
+      </c>
+      <c r="H6">
+        <v>100</v>
+      </c>
+      <c r="I6">
+        <v>7.0709999999999997</v>
+      </c>
+      <c r="J6">
+        <v>100</v>
+      </c>
+      <c r="K6">
+        <v>12.648999999999999</v>
+      </c>
+      <c r="L6">
+        <v>100</v>
+      </c>
+      <c r="M6">
+        <v>5.1559999999999997</v>
+      </c>
+      <c r="N6">
+        <v>66.67</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7">
+        <v>1.1679999999999999</v>
+      </c>
+      <c r="D7">
+        <v>40</v>
+      </c>
+      <c r="E7">
+        <v>0.81</v>
+      </c>
+      <c r="F7">
+        <v>60</v>
+      </c>
+      <c r="G7">
+        <v>0.186</v>
+      </c>
+      <c r="H7">
+        <v>60</v>
+      </c>
+      <c r="I7">
+        <v>-1.1160000000000001</v>
+      </c>
+      <c r="J7">
+        <v>40</v>
+      </c>
+      <c r="K7">
+        <v>-2.5070000000000001</v>
+      </c>
+      <c r="L7">
+        <v>20</v>
+      </c>
+      <c r="M7">
+        <v>-2.4409999999999998</v>
+      </c>
+      <c r="N7">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>1.288</v>
+      </c>
+      <c r="D8">
+        <v>100</v>
+      </c>
+      <c r="E8">
+        <v>0.86</v>
+      </c>
+      <c r="F8">
+        <v>100</v>
+      </c>
+      <c r="G8">
+        <v>1.661</v>
+      </c>
+      <c r="H8">
+        <v>100</v>
+      </c>
+      <c r="I8">
+        <v>2.7719999999999998</v>
+      </c>
+      <c r="J8">
+        <v>100</v>
+      </c>
+      <c r="K8">
+        <v>17.22</v>
+      </c>
+      <c r="L8">
+        <v>100</v>
+      </c>
+      <c r="M8">
+        <v>19.041</v>
+      </c>
+      <c r="N8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="C9">
+        <v>-1.0649999999999999</v>
+      </c>
+      <c r="D9">
+        <v>50</v>
+      </c>
+      <c r="E9">
+        <v>-3.97</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>-4.1310000000000002</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>-2.4729999999999999</v>
+      </c>
+      <c r="J9">
+        <v>50</v>
+      </c>
+      <c r="K9">
+        <v>2.1720000000000002</v>
+      </c>
+      <c r="L9">
+        <v>50</v>
+      </c>
+      <c r="M9">
+        <v>-9.6709999999999994</v>
+      </c>
+      <c r="N9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10">
+        <v>22</v>
+      </c>
+      <c r="C10">
+        <v>2.3149999999999999</v>
+      </c>
+      <c r="D10">
+        <v>59.09</v>
+      </c>
+      <c r="E10">
+        <v>1.8440000000000001</v>
+      </c>
+      <c r="F10">
+        <v>54.55</v>
+      </c>
+      <c r="G10">
+        <v>2.6669999999999998</v>
+      </c>
+      <c r="H10">
+        <v>54.55</v>
+      </c>
+      <c r="I10">
+        <v>2.4910000000000001</v>
+      </c>
+      <c r="J10">
+        <v>54.55</v>
+      </c>
+      <c r="K10">
+        <v>4.9059999999999997</v>
+      </c>
+      <c r="L10">
+        <v>54.55</v>
+      </c>
+      <c r="M10">
+        <v>5.9269999999999996</v>
+      </c>
+      <c r="N10">
+        <v>63.64</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B368DC99-EBF8-4A00-802D-AA0169179304}">
   <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -8184,7 +8399,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7692A300-0829-47F4-83C8-0244C496CBE7}">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -8250,45 +8465,40 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03F0E254-FFBE-404B-9923-6F5E2BA45FC0}">
-  <dimension ref="A1:N75"/>
+  <dimension ref="A2:N75"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="21" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" style="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.7109375" style="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="22.42578125" style="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="23.42578125" style="12" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.5703125" style="12"/>
+    <col min="1" max="1" width="13.42578125" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="22.42578125" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="23.42578125" style="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.5703125" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F1" s="13"/>
-    </row>
     <row r="2" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="D2" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="E2" s="16" t="s">
+      <c r="E2" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="F2" s="16" t="s">
+      <c r="F2" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
     </row>
     <row r="3" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="12" t="s">
         <v>45</v>
       </c>
       <c r="B3" s="7">
@@ -8310,7 +8520,7 @@
       </c>
     </row>
     <row r="4" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="12" t="s">
         <v>46</v>
       </c>
       <c r="B4" s="7">
@@ -8332,7 +8542,7 @@
       </c>
     </row>
     <row r="5" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="12" t="s">
         <v>47</v>
       </c>
       <c r="B5" s="7">
@@ -8354,7 +8564,7 @@
       </c>
     </row>
     <row r="6" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="14" t="s">
         <v>50</v>
       </c>
       <c r="B6" s="9">
@@ -8369,17 +8579,16 @@
         <f t="shared" si="2"/>
         <v>33</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="68">
         <f>SUM(E3:E5)</f>
         <v>8250</v>
       </c>
-      <c r="F6" s="18">
+      <c r="F6" s="70">
         <v>1</v>
       </c>
-      <c r="K6" s="13"/>
     </row>
     <row r="7" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="11" t="s">
         <v>48</v>
       </c>
       <c r="B7" s="8">
@@ -8394,8 +8603,8 @@
         <f t="shared" si="3"/>
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="E7" s="11"/>
-      <c r="F7" s="19"/>
+      <c r="E7" s="69"/>
+      <c r="F7" s="71"/>
     </row>
     <row r="8" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6"/>
@@ -8442,22 +8651,22 @@
       <c r="N11"/>
     </row>
     <row r="12" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="20">
+      <c r="A12">
         <v>2.3149999999999999</v>
       </c>
-      <c r="B12" s="20">
+      <c r="B12">
         <v>1.8440000000000001</v>
       </c>
-      <c r="C12" s="20">
+      <c r="C12">
         <v>2.6669999999999998</v>
       </c>
-      <c r="D12" s="20">
+      <c r="D12">
         <v>2.4910000000000001</v>
       </c>
-      <c r="E12" s="20">
+      <c r="E12">
         <v>4.9059999999999997</v>
       </c>
-      <c r="F12" s="20">
+      <c r="F12">
         <v>5.9269999999999996</v>
       </c>
       <c r="G12"/>
@@ -8470,12 +8679,12 @@
       <c r="N12"/>
     </row>
     <row r="13" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="20"/>
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
+      <c r="A13"/>
+      <c r="B13"/>
+      <c r="C13"/>
+      <c r="D13"/>
+      <c r="E13"/>
+      <c r="F13"/>
       <c r="G13"/>
       <c r="H13"/>
       <c r="I13"/>
@@ -8492,10 +8701,10 @@
       <c r="B14" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
+      <c r="C14"/>
+      <c r="D14"/>
+      <c r="E14"/>
+      <c r="F14"/>
       <c r="G14"/>
       <c r="H14"/>
       <c r="I14"/>
@@ -8550,22 +8759,22 @@
       <c r="N16"/>
     </row>
     <row r="17" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="20">
+      <c r="A17">
         <v>59.09</v>
       </c>
-      <c r="B17" s="20">
+      <c r="B17">
         <v>54.55</v>
       </c>
-      <c r="C17" s="20">
+      <c r="C17">
         <v>54.55</v>
       </c>
-      <c r="D17" s="20">
+      <c r="D17">
         <v>54.55</v>
       </c>
-      <c r="E17" s="20">
+      <c r="E17">
         <v>54.55</v>
       </c>
-      <c r="F17" s="20">
+      <c r="F17">
         <v>63.64</v>
       </c>
       <c r="G17"/>
@@ -8621,13 +8830,13 @@
       <c r="A20" s="3">
         <v>1</v>
       </c>
-      <c r="B20" s="22">
+      <c r="B20" s="3">
         <v>2.3149999999999999</v>
       </c>
-      <c r="C20" s="22">
+      <c r="C20" s="3">
         <v>59.09</v>
       </c>
-      <c r="D20" s="22">
+      <c r="D20" s="3">
         <v>50</v>
       </c>
       <c r="E20"/>
@@ -8645,13 +8854,13 @@
       <c r="A21" s="3">
         <v>2</v>
       </c>
-      <c r="B21" s="22">
+      <c r="B21" s="3">
         <v>1.8440000000000001</v>
       </c>
-      <c r="C21" s="22">
+      <c r="C21" s="3">
         <v>54.55</v>
       </c>
-      <c r="D21" s="22">
+      <c r="D21" s="3">
         <v>50</v>
       </c>
       <c r="E21"/>
@@ -8669,13 +8878,13 @@
       <c r="A22" s="3">
         <v>3</v>
       </c>
-      <c r="B22" s="22">
+      <c r="B22" s="3">
         <v>2.6669999999999998</v>
       </c>
-      <c r="C22" s="22">
+      <c r="C22" s="3">
         <v>54.55</v>
       </c>
-      <c r="D22" s="22">
+      <c r="D22" s="3">
         <v>50</v>
       </c>
       <c r="E22"/>
@@ -8693,13 +8902,13 @@
       <c r="A23" s="3">
         <v>5</v>
       </c>
-      <c r="B23" s="22">
+      <c r="B23" s="3">
         <v>2.4910000000000001</v>
       </c>
-      <c r="C23" s="22">
+      <c r="C23" s="3">
         <v>54.55</v>
       </c>
-      <c r="D23" s="22">
+      <c r="D23" s="3">
         <v>50</v>
       </c>
       <c r="E23"/>
@@ -8710,13 +8919,13 @@
       <c r="A24" s="3">
         <v>10</v>
       </c>
-      <c r="B24" s="22">
+      <c r="B24" s="3">
         <v>4.9059999999999997</v>
       </c>
-      <c r="C24" s="22">
+      <c r="C24" s="3">
         <v>54.55</v>
       </c>
-      <c r="D24" s="22">
+      <c r="D24" s="3">
         <v>50</v>
       </c>
     </row>
@@ -8724,13 +8933,13 @@
       <c r="A25" s="3">
         <v>21</v>
       </c>
-      <c r="B25" s="22">
+      <c r="B25" s="3">
         <v>5.9269999999999996</v>
       </c>
-      <c r="C25" s="22">
+      <c r="C25" s="3">
         <v>63.64</v>
       </c>
-      <c r="D25" s="22">
+      <c r="D25" s="3">
         <v>50</v>
       </c>
     </row>
@@ -8798,209 +9007,209 @@
       </c>
     </row>
     <row r="44" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="21" t="s">
+      <c r="A44" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="B44" s="20">
+      <c r="B44">
         <v>1.1539999999999999</v>
       </c>
-      <c r="C44" s="20">
+      <c r="C44">
         <v>1.226</v>
       </c>
-      <c r="D44" s="20">
+      <c r="D44">
         <v>9.0999999999999998E-2</v>
       </c>
-      <c r="E44" s="20">
+      <c r="E44">
         <v>-0.247</v>
       </c>
-      <c r="F44" s="20">
+      <c r="F44">
         <v>-1.7989999999999999</v>
       </c>
-      <c r="G44" s="20">
+      <c r="G44">
         <v>-6.0869999999999997</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="21" t="s">
+      <c r="A45" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="B45" s="20">
+      <c r="B45">
         <v>-0.57999999999999996</v>
       </c>
-      <c r="C45" s="20">
+      <c r="C45">
         <v>0.13300000000000001</v>
       </c>
-      <c r="D45" s="20">
+      <c r="D45">
         <v>-0.64500000000000002</v>
       </c>
-      <c r="E45" s="20">
+      <c r="E45">
         <v>-0.53900000000000003</v>
       </c>
-      <c r="F45" s="20">
+      <c r="F45">
         <v>1.611</v>
       </c>
-      <c r="G45" s="20">
+      <c r="G45">
         <v>15.06</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A46" s="21" t="s">
+      <c r="A46" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="B46" s="20">
+      <c r="B46">
         <v>-1.1359999999999999</v>
       </c>
-      <c r="C46" s="20">
+      <c r="C46">
         <v>-1.0109999999999999</v>
       </c>
-      <c r="D46" s="20">
+      <c r="D46">
         <v>-0.86299999999999999</v>
       </c>
-      <c r="E46" s="20">
+      <c r="E46">
         <v>-0.21299999999999999</v>
       </c>
-      <c r="F46" s="20">
+      <c r="F46">
         <v>2.76</v>
       </c>
-      <c r="G46" s="20">
+      <c r="G46">
         <v>7.1580000000000004</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A47" s="21" t="s">
+      <c r="A47" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B47" s="20">
+      <c r="B47">
         <v>32.093000000000004</v>
       </c>
-      <c r="C47" s="20">
+      <c r="C47">
         <v>33.332999999999998</v>
       </c>
-      <c r="D47" s="20">
+      <c r="D47">
         <v>53.444000000000003</v>
       </c>
-      <c r="E47" s="20">
+      <c r="E47">
         <v>44.877000000000002</v>
       </c>
-      <c r="F47" s="20">
+      <c r="F47">
         <v>51.631</v>
       </c>
-      <c r="G47" s="20">
+      <c r="G47">
         <v>63.975999999999999</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A48" s="21" t="s">
+      <c r="A48" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B48" s="20">
+      <c r="B48">
         <v>5.3710000000000004</v>
       </c>
-      <c r="C48" s="20">
+      <c r="C48">
         <v>3.0259999999999998</v>
       </c>
-      <c r="D48" s="20">
+      <c r="D48">
         <v>5.2670000000000003</v>
       </c>
-      <c r="E48" s="20">
+      <c r="E48">
         <v>7.0709999999999997</v>
       </c>
-      <c r="F48" s="20">
+      <c r="F48">
         <v>12.648999999999999</v>
       </c>
-      <c r="G48" s="20">
+      <c r="G48">
         <v>5.1559999999999997</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A49" s="21" t="s">
+      <c r="A49" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="B49" s="20">
+      <c r="B49">
         <v>1.1679999999999999</v>
       </c>
-      <c r="C49" s="20">
+      <c r="C49">
         <v>0.81</v>
       </c>
-      <c r="D49" s="20">
+      <c r="D49">
         <v>0.186</v>
       </c>
-      <c r="E49" s="20">
+      <c r="E49">
         <v>-1.1160000000000001</v>
       </c>
-      <c r="F49" s="20">
+      <c r="F49">
         <v>-2.5070000000000001</v>
       </c>
-      <c r="G49" s="20">
+      <c r="G49">
         <v>-2.4409999999999998</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A50" s="21" t="s">
+      <c r="A50" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B50" s="20">
+      <c r="B50">
         <v>1.288</v>
       </c>
-      <c r="C50" s="20">
+      <c r="C50">
         <v>0.86</v>
       </c>
-      <c r="D50" s="20">
+      <c r="D50">
         <v>1.661</v>
       </c>
-      <c r="E50" s="20">
+      <c r="E50">
         <v>2.7719999999999998</v>
       </c>
-      <c r="F50" s="20">
+      <c r="F50">
         <v>17.22</v>
       </c>
-      <c r="G50" s="20">
+      <c r="G50">
         <v>19.041</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A51" s="21" t="s">
+      <c r="A51" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B51" s="20">
+      <c r="B51">
         <v>-1.0649999999999999</v>
       </c>
-      <c r="C51" s="20">
+      <c r="C51">
         <v>-3.97</v>
       </c>
-      <c r="D51" s="20">
+      <c r="D51">
         <v>-4.1310000000000002</v>
       </c>
-      <c r="E51" s="20">
+      <c r="E51">
         <v>-2.4729999999999999</v>
       </c>
-      <c r="F51" s="20">
+      <c r="F51">
         <v>2.1720000000000002</v>
       </c>
-      <c r="G51" s="20">
+      <c r="G51">
         <v>-9.6709999999999994</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A52" s="21" t="s">
+      <c r="A52" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="B52" s="20">
+      <c r="B52">
         <v>4.7866249999999999</v>
       </c>
-      <c r="C52" s="20">
+      <c r="C52">
         <v>34.406999999999996</v>
       </c>
-      <c r="D52" s="20">
+      <c r="D52">
         <v>55.010000000000005</v>
       </c>
-      <c r="E52" s="20">
+      <c r="E52">
         <v>50.131999999999998</v>
       </c>
-      <c r="F52" s="20">
+      <c r="F52">
         <v>83.736999999999995</v>
       </c>
-      <c r="G52" s="20">
+      <c r="G52">
         <v>92.192000000000007</v>
       </c>
     </row>
@@ -9015,339 +9224,339 @@
     </row>
     <row r="55" spans="1:8" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="56" spans="1:8" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="23" t="s">
+      <c r="A56" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="B56" s="24" t="s">
+      <c r="B56" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="C56" s="24" t="s">
+      <c r="C56" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="D56" s="24" t="s">
+      <c r="D56" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="E56" s="24" t="s">
+      <c r="E56" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="F56" s="24" t="s">
+      <c r="F56" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="G56" s="24" t="s">
+      <c r="G56" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="H56" s="24" t="s">
+      <c r="H56" s="17" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="25" t="s">
+      <c r="A57" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="B57" s="26">
+      <c r="B57" s="19">
         <v>3</v>
       </c>
-      <c r="C57" s="30">
+      <c r="C57" s="23">
         <v>1.15E-2</v>
       </c>
-      <c r="D57" s="30">
+      <c r="D57" s="23">
         <v>1.23E-2</v>
       </c>
-      <c r="E57" s="30">
+      <c r="E57" s="23">
         <v>8.9999999999999998E-4</v>
       </c>
-      <c r="F57" s="30">
+      <c r="F57" s="23">
         <v>-2.5000000000000001E-3</v>
       </c>
-      <c r="G57" s="30">
+      <c r="G57" s="23">
         <v>-1.8000000000000002E-2</v>
       </c>
-      <c r="H57" s="30">
+      <c r="H57" s="23">
         <v>-6.0899999999999996E-2</v>
       </c>
     </row>
     <row r="58" spans="1:8" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="25" t="s">
+      <c r="A58" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="B58" s="26">
+      <c r="B58" s="19">
         <v>4</v>
       </c>
-      <c r="C58" s="30">
+      <c r="C58" s="23">
         <v>-5.7999999999999996E-3</v>
       </c>
-      <c r="D58" s="30">
+      <c r="D58" s="23">
         <v>1.2999999999999999E-3</v>
       </c>
-      <c r="E58" s="30">
+      <c r="E58" s="23">
         <v>-6.5000000000000006E-3</v>
       </c>
-      <c r="F58" s="30">
+      <c r="F58" s="23">
         <v>-5.4000000000000003E-3</v>
       </c>
-      <c r="G58" s="30">
+      <c r="G58" s="23">
         <v>1.61E-2</v>
       </c>
-      <c r="H58" s="30">
+      <c r="H58" s="23">
         <v>0.15060000000000001</v>
       </c>
     </row>
     <row r="59" spans="1:8" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="25" t="s">
+      <c r="A59" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="B59" s="26">
+      <c r="B59" s="19">
         <v>3</v>
       </c>
-      <c r="C59" s="30">
+      <c r="C59" s="23">
         <v>-1.1399999999999999E-2</v>
       </c>
-      <c r="D59" s="30">
+      <c r="D59" s="23">
         <v>-1.01E-2</v>
       </c>
-      <c r="E59" s="30">
+      <c r="E59" s="23">
         <v>-8.6E-3</v>
       </c>
-      <c r="F59" s="30">
+      <c r="F59" s="23">
         <v>-2.0999999999999999E-3</v>
       </c>
-      <c r="G59" s="30">
+      <c r="G59" s="23">
         <v>2.76E-2</v>
       </c>
-      <c r="H59" s="30">
+      <c r="H59" s="23">
         <v>7.1599999999999997E-2</v>
       </c>
     </row>
     <row r="60" spans="1:8" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="25" t="s">
+      <c r="A60" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="B60" s="26">
+      <c r="B60" s="19">
         <v>1</v>
       </c>
-      <c r="C60" s="30">
+      <c r="C60" s="23">
         <v>0.32090000000000002</v>
       </c>
-      <c r="D60" s="30">
+      <c r="D60" s="23">
         <v>0.33329999999999999</v>
       </c>
-      <c r="E60" s="30">
+      <c r="E60" s="23">
         <v>0.53439999999999999</v>
       </c>
-      <c r="F60" s="30">
+      <c r="F60" s="23">
         <v>0.44880000000000003</v>
       </c>
-      <c r="G60" s="30">
+      <c r="G60" s="23">
         <v>0.51629999999999998</v>
       </c>
-      <c r="H60" s="30">
+      <c r="H60" s="23">
         <v>0.63979999999999992</v>
       </c>
     </row>
     <row r="61" spans="1:8" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="25" t="s">
+      <c r="A61" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="B61" s="26">
+      <c r="B61" s="19">
         <v>3</v>
       </c>
-      <c r="C61" s="30">
+      <c r="C61" s="23">
         <v>5.3699999999999998E-2</v>
       </c>
-      <c r="D61" s="30">
+      <c r="D61" s="23">
         <v>3.0299999999999997E-2</v>
       </c>
-      <c r="E61" s="30">
+      <c r="E61" s="23">
         <v>5.2699999999999997E-2</v>
       </c>
-      <c r="F61" s="30">
+      <c r="F61" s="23">
         <v>7.0699999999999999E-2</v>
       </c>
-      <c r="G61" s="30">
+      <c r="G61" s="23">
         <v>0.1265</v>
       </c>
-      <c r="H61" s="30">
+      <c r="H61" s="23">
         <v>5.16E-2</v>
       </c>
     </row>
     <row r="62" spans="1:8" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="25" t="s">
+      <c r="A62" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="B62" s="26">
+      <c r="B62" s="19">
         <v>5</v>
       </c>
-      <c r="C62" s="30">
+      <c r="C62" s="23">
         <v>1.1699999999999999E-2</v>
       </c>
-      <c r="D62" s="30">
+      <c r="D62" s="23">
         <v>8.1000000000000013E-3</v>
       </c>
-      <c r="E62" s="30">
+      <c r="E62" s="23">
         <v>1.9E-3</v>
       </c>
-      <c r="F62" s="30">
+      <c r="F62" s="23">
         <v>-1.1200000000000002E-2</v>
       </c>
-      <c r="G62" s="30">
+      <c r="G62" s="23">
         <v>-2.5099999999999997E-2</v>
       </c>
-      <c r="H62" s="30">
+      <c r="H62" s="23">
         <v>-2.4399999999999998E-2</v>
       </c>
     </row>
     <row r="63" spans="1:8" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="25" t="s">
+      <c r="A63" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="B63" s="26">
+      <c r="B63" s="19">
         <v>1</v>
       </c>
-      <c r="C63" s="30">
+      <c r="C63" s="23">
         <v>1.29E-2</v>
       </c>
-      <c r="D63" s="30">
+      <c r="D63" s="23">
         <v>8.6E-3</v>
       </c>
-      <c r="E63" s="30">
+      <c r="E63" s="23">
         <v>1.66E-2</v>
       </c>
-      <c r="F63" s="30">
+      <c r="F63" s="23">
         <v>2.7699999999999999E-2</v>
       </c>
-      <c r="G63" s="30">
+      <c r="G63" s="23">
         <v>0.17219999999999999</v>
       </c>
-      <c r="H63" s="30">
+      <c r="H63" s="23">
         <v>0.19039999999999999</v>
       </c>
     </row>
     <row r="64" spans="1:8" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="25" t="s">
+      <c r="A64" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B64" s="26">
+      <c r="B64" s="19">
         <v>2</v>
       </c>
-      <c r="C64" s="30">
+      <c r="C64" s="23">
         <v>-1.0700000000000001E-2</v>
       </c>
-      <c r="D64" s="30">
+      <c r="D64" s="23">
         <v>-3.9699999999999999E-2</v>
       </c>
-      <c r="E64" s="30">
+      <c r="E64" s="23">
         <v>-4.1299999999999996E-2</v>
       </c>
-      <c r="F64" s="30">
+      <c r="F64" s="23">
         <v>-2.4700000000000003E-2</v>
       </c>
-      <c r="G64" s="30">
+      <c r="G64" s="23">
         <v>2.1700000000000001E-2</v>
       </c>
-      <c r="H64" s="30">
+      <c r="H64" s="23">
         <v>-9.6699999999999994E-2</v>
       </c>
     </row>
     <row r="65" spans="1:8" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="27" t="s">
+      <c r="A65" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="B65" s="28">
+      <c r="B65" s="21">
         <v>22</v>
       </c>
-      <c r="C65" s="31">
+      <c r="C65" s="24">
         <v>2.3199999999999998E-2</v>
       </c>
-      <c r="D65" s="31">
+      <c r="D65" s="24">
         <v>1.84E-2</v>
       </c>
-      <c r="E65" s="31">
+      <c r="E65" s="24">
         <v>2.6699999999999998E-2</v>
       </c>
-      <c r="F65" s="31">
+      <c r="F65" s="24">
         <v>2.4900000000000002E-2</v>
       </c>
-      <c r="G65" s="31">
+      <c r="G65" s="24">
         <v>4.9100000000000005E-2</v>
       </c>
-      <c r="H65" s="31">
+      <c r="H65" s="24">
         <v>5.9299999999999999E-2</v>
       </c>
     </row>
     <row r="67" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C67" s="29"/>
-      <c r="D67" s="29"/>
-      <c r="E67" s="29"/>
-      <c r="F67" s="29"/>
-      <c r="G67" s="29"/>
-      <c r="H67" s="29"/>
+      <c r="C67" s="22"/>
+      <c r="D67" s="22"/>
+      <c r="E67" s="22"/>
+      <c r="F67" s="22"/>
+      <c r="G67" s="22"/>
+      <c r="H67" s="22"/>
     </row>
     <row r="68" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C68" s="29"/>
-      <c r="D68" s="29"/>
-      <c r="E68" s="29"/>
-      <c r="F68" s="29"/>
-      <c r="G68" s="29">
+      <c r="C68" s="22"/>
+      <c r="D68" s="22"/>
+      <c r="E68" s="22"/>
+      <c r="F68" s="22"/>
+      <c r="G68" s="22">
         <f>G65-F65</f>
         <v>2.4200000000000003E-2</v>
       </c>
-      <c r="H68" s="29"/>
+      <c r="H68" s="22"/>
     </row>
     <row r="69" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C69" s="29"/>
-      <c r="D69" s="29"/>
-      <c r="E69" s="29"/>
-      <c r="F69" s="29"/>
-      <c r="G69" s="29"/>
-      <c r="H69" s="29"/>
+      <c r="C69" s="22"/>
+      <c r="D69" s="22"/>
+      <c r="E69" s="22"/>
+      <c r="F69" s="22"/>
+      <c r="G69" s="22"/>
+      <c r="H69" s="22"/>
     </row>
     <row r="70" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C70" s="29"/>
-      <c r="D70" s="29"/>
-      <c r="E70" s="29"/>
-      <c r="F70" s="29"/>
-      <c r="G70" s="29"/>
-      <c r="H70" s="29"/>
+      <c r="C70" s="22"/>
+      <c r="D70" s="22"/>
+      <c r="E70" s="22"/>
+      <c r="F70" s="22"/>
+      <c r="G70" s="22"/>
+      <c r="H70" s="22"/>
     </row>
     <row r="71" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C71" s="29"/>
-      <c r="D71" s="29"/>
-      <c r="E71" s="29"/>
-      <c r="F71" s="29"/>
-      <c r="G71" s="29"/>
-      <c r="H71" s="29"/>
+      <c r="C71" s="22"/>
+      <c r="D71" s="22"/>
+      <c r="E71" s="22"/>
+      <c r="F71" s="22"/>
+      <c r="G71" s="22"/>
+      <c r="H71" s="22"/>
     </row>
     <row r="72" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C72" s="29"/>
-      <c r="D72" s="29"/>
-      <c r="E72" s="29"/>
-      <c r="F72" s="29"/>
-      <c r="G72" s="29"/>
-      <c r="H72" s="29"/>
+      <c r="C72" s="22"/>
+      <c r="D72" s="22"/>
+      <c r="E72" s="22"/>
+      <c r="F72" s="22"/>
+      <c r="G72" s="22"/>
+      <c r="H72" s="22"/>
     </row>
     <row r="73" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C73" s="29"/>
-      <c r="D73" s="29"/>
-      <c r="E73" s="29"/>
-      <c r="F73" s="29"/>
-      <c r="G73" s="29"/>
-      <c r="H73" s="29"/>
+      <c r="C73" s="22"/>
+      <c r="D73" s="22"/>
+      <c r="E73" s="22"/>
+      <c r="F73" s="22"/>
+      <c r="G73" s="22"/>
+      <c r="H73" s="22"/>
     </row>
     <row r="74" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C74" s="29"/>
-      <c r="D74" s="29"/>
-      <c r="E74" s="29"/>
-      <c r="F74" s="29"/>
-      <c r="G74" s="29"/>
-      <c r="H74" s="29"/>
+      <c r="C74" s="22"/>
+      <c r="D74" s="22"/>
+      <c r="E74" s="22"/>
+      <c r="F74" s="22"/>
+      <c r="G74" s="22"/>
+      <c r="H74" s="22"/>
     </row>
     <row r="75" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C75" s="29"/>
-      <c r="D75" s="29"/>
-      <c r="E75" s="29"/>
-      <c r="F75" s="29"/>
-      <c r="G75" s="29"/>
-      <c r="H75" s="29"/>
+      <c r="C75" s="22"/>
+      <c r="D75" s="22"/>
+      <c r="E75" s="22"/>
+      <c r="F75" s="22"/>
+      <c r="G75" s="22"/>
+      <c r="H75" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -9359,120 +9568,120 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7ABD143F-FD3E-489B-9763-A634E4AA9F53}">
   <dimension ref="A2:C10"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12" style="32" customWidth="1"/>
-    <col min="2" max="4" width="18" style="32" customWidth="1"/>
-    <col min="5" max="16384" width="8.7109375" style="32"/>
+    <col min="1" max="1" width="12" style="25" customWidth="1"/>
+    <col min="2" max="4" width="18" style="25" customWidth="1"/>
+    <col min="5" max="16384" width="8.7109375" style="25"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="26" t="s">
         <v>77</v>
       </c>
-      <c r="C2" s="33" t="s">
+      <c r="C2" s="26" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="34" t="s">
+      <c r="A3" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="35">
-        <f>VLOOKUP(A3,[2]Raw_Data!$A$5:$G$15,3,FALSE())</f>
+      <c r="B3" s="28">
+        <f>VLOOKUP(A3,[1]Raw_Data!$A$5:$G$15,3,FALSE())</f>
         <v>100</v>
       </c>
-      <c r="C3" s="36">
+      <c r="C3" s="29">
         <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="34" t="s">
+      <c r="A4" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="35">
-        <f>VLOOKUP(A4,[2]Raw_Data!$A$5:$G$15,3,FALSE())</f>
+      <c r="B4" s="28">
+        <f>VLOOKUP(A4,[1]Raw_Data!$A$5:$G$15,3,FALSE())</f>
         <v>81.25</v>
       </c>
-      <c r="C4" s="36">
+      <c r="C4" s="29">
         <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="34" t="s">
+      <c r="A5" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="35">
-        <f>VLOOKUP(A5,[2]Raw_Data!$A$5:$G$15,3,FALSE())</f>
+      <c r="B5" s="28">
+        <f>VLOOKUP(A5,[1]Raw_Data!$A$5:$G$15,3,FALSE())</f>
         <v>75</v>
       </c>
-      <c r="C5" s="36">
+      <c r="C5" s="29">
         <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="34" t="s">
+      <c r="A6" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="35">
-        <f>VLOOKUP(A6,[2]Raw_Data!$A$5:$G$15,3,FALSE())</f>
+      <c r="B6" s="28">
+        <f>VLOOKUP(A6,[1]Raw_Data!$A$5:$G$15,3,FALSE())</f>
         <v>71.430000000000007</v>
       </c>
-      <c r="C6" s="36">
+      <c r="C6" s="29">
         <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="34" t="s">
+      <c r="A7" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="35">
-        <f>VLOOKUP(A7,[2]Raw_Data!$A$5:$G$15,3,FALSE())</f>
+      <c r="B7" s="28">
+        <f>VLOOKUP(A7,[1]Raw_Data!$A$5:$G$15,3,FALSE())</f>
         <v>66.67</v>
       </c>
-      <c r="C7" s="36">
+      <c r="C7" s="29">
         <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="34" t="s">
+      <c r="A8" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="35">
-        <f>VLOOKUP(A8,[2]Raw_Data!$A$5:$G$15,3,FALSE())</f>
+      <c r="B8" s="28">
+        <f>VLOOKUP(A8,[1]Raw_Data!$A$5:$G$15,3,FALSE())</f>
         <v>66.67</v>
       </c>
-      <c r="C8" s="36">
+      <c r="C8" s="29">
         <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="34" t="s">
+      <c r="A9" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="35">
-        <f>VLOOKUP(A9,[2]Raw_Data!$A$5:$G$15,3,FALSE())</f>
+      <c r="B9" s="28">
+        <f>VLOOKUP(A9,[1]Raw_Data!$A$5:$G$15,3,FALSE())</f>
         <v>33.33</v>
       </c>
-      <c r="C9" s="36">
+      <c r="C9" s="29">
         <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="34" t="s">
+      <c r="A10" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="35">
-        <f>VLOOKUP(A10,[2]Raw_Data!$A$5:$G$15,3,FALSE())</f>
+      <c r="B10" s="28">
+        <f>VLOOKUP(A10,[1]Raw_Data!$A$5:$G$15,3,FALSE())</f>
         <v>0</v>
       </c>
-      <c r="C10" s="36">
+      <c r="C10" s="29">
         <v>85</v>
       </c>
     </row>
@@ -9483,144 +9692,144 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FBAE775-042E-492A-B18F-94EC939471D4}">
   <dimension ref="A2:C12"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12" style="32" customWidth="1"/>
-    <col min="2" max="4" width="18" style="32" customWidth="1"/>
-    <col min="5" max="16384" width="8.7109375" style="32"/>
+    <col min="1" max="1" width="12" style="25" customWidth="1"/>
+    <col min="2" max="4" width="18" style="25" customWidth="1"/>
+    <col min="5" max="16384" width="8.7109375" style="25"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="26" t="s">
         <v>79</v>
       </c>
-      <c r="C2" s="33" t="s">
+      <c r="C2" s="26" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="34" t="s">
+      <c r="A3" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="35">
-        <f>VLOOKUP(A3,[2]Raw_Data!$A$5:$G$15,6,FALSE())</f>
+      <c r="B3" s="28">
+        <f>VLOOKUP(A3,[1]Raw_Data!$A$5:$G$15,6,FALSE())</f>
         <v>2.09</v>
       </c>
-      <c r="C3" s="37">
+      <c r="C3" s="30">
         <v>2.27</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="34" t="s">
+      <c r="A4" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="35">
-        <f>VLOOKUP(A4,[2]Raw_Data!$A$5:$G$15,6,FALSE())</f>
+      <c r="B4" s="28">
+        <f>VLOOKUP(A4,[1]Raw_Data!$A$5:$G$15,6,FALSE())</f>
         <v>1.57</v>
       </c>
-      <c r="C4" s="37">
+      <c r="C4" s="30">
         <v>2.27</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="34" t="s">
+      <c r="A5" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="35">
-        <f>VLOOKUP(A5,[2]Raw_Data!$A$5:$G$15,6,FALSE())</f>
+      <c r="B5" s="28">
+        <f>VLOOKUP(A5,[1]Raw_Data!$A$5:$G$15,6,FALSE())</f>
         <v>1.54</v>
       </c>
-      <c r="C5" s="37">
+      <c r="C5" s="30">
         <v>2.27</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="34" t="s">
+      <c r="A6" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="35">
-        <f>VLOOKUP(A6,[2]Raw_Data!$A$5:$G$15,6,FALSE())</f>
+      <c r="B6" s="28">
+        <f>VLOOKUP(A6,[1]Raw_Data!$A$5:$G$15,6,FALSE())</f>
         <v>1.44</v>
       </c>
-      <c r="C6" s="37">
+      <c r="C6" s="30">
         <v>2.27</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="34" t="s">
+      <c r="A7" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="35">
-        <f>VLOOKUP(A7,[2]Raw_Data!$A$5:$G$15,6,FALSE())</f>
+      <c r="B7" s="28">
+        <f>VLOOKUP(A7,[1]Raw_Data!$A$5:$G$15,6,FALSE())</f>
         <v>1.19</v>
       </c>
-      <c r="C7" s="37">
+      <c r="C7" s="30">
         <v>2.27</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="34" t="s">
+      <c r="A8" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="35">
-        <f>VLOOKUP(A8,[2]Raw_Data!$A$5:$G$15,6,FALSE())</f>
+      <c r="B8" s="28">
+        <f>VLOOKUP(A8,[1]Raw_Data!$A$5:$G$15,6,FALSE())</f>
         <v>1.18</v>
       </c>
-      <c r="C8" s="37">
+      <c r="C8" s="30">
         <v>2.27</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="34" t="s">
+      <c r="A9" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="35">
-        <f>VLOOKUP(A9,[2]Raw_Data!$A$5:$G$15,6,FALSE())</f>
+      <c r="B9" s="28">
+        <f>VLOOKUP(A9,[1]Raw_Data!$A$5:$G$15,6,FALSE())</f>
         <v>1.02</v>
       </c>
-      <c r="C9" s="37">
+      <c r="C9" s="30">
         <v>2.27</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="34" t="s">
+      <c r="A10" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="35">
-        <f>VLOOKUP(A10,[2]Raw_Data!$A$5:$G$15,6,FALSE())</f>
+      <c r="B10" s="28">
+        <f>VLOOKUP(A10,[1]Raw_Data!$A$5:$G$15,6,FALSE())</f>
         <v>0.91</v>
       </c>
-      <c r="C10" s="37">
+      <c r="C10" s="30">
         <v>2.27</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="34" t="s">
+      <c r="A11" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="35">
-        <f>VLOOKUP(A11,[2]Raw_Data!$A$5:$G$15,6,FALSE())</f>
+      <c r="B11" s="28">
+        <f>VLOOKUP(A11,[1]Raw_Data!$A$5:$G$15,6,FALSE())</f>
         <v>0.66</v>
       </c>
-      <c r="C11" s="37">
+      <c r="C11" s="30">
         <v>2.27</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="34" t="s">
+      <c r="A12" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="35">
-        <f>VLOOKUP(A12,[2]Raw_Data!$A$5:$G$15,6,FALSE())</f>
+      <c r="B12" s="28">
+        <f>VLOOKUP(A12,[1]Raw_Data!$A$5:$G$15,6,FALSE())</f>
         <v>-0.71</v>
       </c>
-      <c r="C12" s="37">
+      <c r="C12" s="30">
         <v>2.27</v>
       </c>
     </row>
@@ -9645,202 +9854,202 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="46" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="64" t="s">
+      <c r="B1" s="47" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="63" t="s">
+      <c r="C1" s="46" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="63" t="s">
+      <c r="D1" s="46" t="s">
         <v>93</v>
       </c>
-      <c r="E1" s="64" t="s">
+      <c r="E1" s="47" t="s">
         <v>94</v>
       </c>
-      <c r="F1" s="63" t="s">
+      <c r="F1" s="46" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="32" t="s">
         <v>96</v>
       </c>
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="41" t="s">
         <v>97</v>
       </c>
-      <c r="C2" s="40" t="s">
+      <c r="C2" s="32" t="s">
         <v>98</v>
       </c>
-      <c r="D2" s="40" t="s">
+      <c r="D2" s="32" t="s">
         <v>99</v>
       </c>
-      <c r="E2" s="55" t="s">
+      <c r="E2" s="41" t="s">
         <v>100</v>
       </c>
-      <c r="F2" s="40" t="s">
+      <c r="F2" s="32" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="32" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="55" t="s">
+      <c r="B3" s="41" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="32" t="s">
         <v>104</v>
       </c>
-      <c r="D3" s="40" t="s">
+      <c r="D3" s="32" t="s">
         <v>104</v>
       </c>
-      <c r="E3" s="55" t="s">
+      <c r="E3" s="41" t="s">
         <v>99</v>
       </c>
-      <c r="F3" s="40" t="s">
+      <c r="F3" s="32" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="32" t="s">
         <v>106</v>
       </c>
-      <c r="B4" s="55" t="s">
+      <c r="B4" s="41" t="s">
         <v>104</v>
       </c>
-      <c r="C4" s="40" t="s">
+      <c r="C4" s="32" t="s">
         <v>98</v>
       </c>
-      <c r="D4" s="40" t="s">
+      <c r="D4" s="32" t="s">
         <v>107</v>
       </c>
-      <c r="E4" s="55" t="s">
+      <c r="E4" s="41" t="s">
         <v>108</v>
       </c>
-      <c r="F4" s="40" t="s">
+      <c r="F4" s="32" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="40" t="s">
+      <c r="A5" s="32" t="s">
         <v>109</v>
       </c>
-      <c r="B5" s="55" t="s">
+      <c r="B5" s="41" t="s">
         <v>104</v>
       </c>
-      <c r="C5" s="40" t="s">
+      <c r="C5" s="32" t="s">
         <v>104</v>
       </c>
-      <c r="D5" s="40" t="s">
+      <c r="D5" s="32" t="s">
         <v>104</v>
       </c>
-      <c r="E5" s="55" t="s">
+      <c r="E5" s="41" t="s">
         <v>104</v>
       </c>
-      <c r="F5" s="40" t="s">
+      <c r="F5" s="32" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="40" t="s">
+      <c r="A6" s="32" t="s">
         <v>110</v>
       </c>
-      <c r="B6" s="55" t="s">
+      <c r="B6" s="41" t="s">
         <v>111</v>
       </c>
-      <c r="C6" s="40" t="s">
+      <c r="C6" s="32" t="s">
         <v>98</v>
       </c>
-      <c r="D6" s="40" t="s">
+      <c r="D6" s="32" t="s">
         <v>104</v>
       </c>
-      <c r="E6" s="55" t="s">
+      <c r="E6" s="41" t="s">
         <v>104</v>
       </c>
-      <c r="F6" s="40" t="s">
+      <c r="F6" s="32" t="s">
         <v>200</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="40" t="s">
+      <c r="A7" s="32" t="s">
         <v>112</v>
       </c>
-      <c r="B7" s="55" t="s">
+      <c r="B7" s="41" t="s">
         <v>104</v>
       </c>
-      <c r="C7" s="40" t="s">
+      <c r="C7" s="32" t="s">
         <v>99</v>
       </c>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="32" t="s">
         <v>113</v>
       </c>
-      <c r="E7" s="55" t="s">
+      <c r="E7" s="41" t="s">
         <v>104</v>
       </c>
-      <c r="F7" s="40" t="s">
+      <c r="F7" s="32" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="40" t="s">
+      <c r="A8" s="32" t="s">
         <v>115</v>
       </c>
-      <c r="B8" s="55" t="s">
+      <c r="B8" s="41" t="s">
         <v>104</v>
       </c>
-      <c r="C8" s="40" t="s">
+      <c r="C8" s="32" t="s">
         <v>104</v>
       </c>
-      <c r="D8" s="40" t="s">
+      <c r="D8" s="32" t="s">
         <v>104</v>
       </c>
-      <c r="E8" s="55" t="s">
+      <c r="E8" s="41" t="s">
         <v>104</v>
       </c>
-      <c r="F8" s="40" t="s">
+      <c r="F8" s="32" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="40" t="s">
+      <c r="A9" s="32" t="s">
         <v>117</v>
       </c>
-      <c r="B9" s="40" t="s">
+      <c r="B9" s="32" t="s">
         <v>118</v>
       </c>
-      <c r="C9" s="40" t="s">
+      <c r="C9" s="32" t="s">
         <v>118</v>
       </c>
-      <c r="D9" s="40" t="s">
+      <c r="D9" s="32" t="s">
         <v>196</v>
       </c>
-      <c r="E9" s="55" t="s">
+      <c r="E9" s="41" t="s">
         <v>197</v>
       </c>
-      <c r="F9" s="40" t="s">
+      <c r="F9" s="32" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="40" t="s">
+      <c r="A10" s="32" t="s">
         <v>201</v>
       </c>
-      <c r="B10" s="55" t="s">
+      <c r="B10" s="41" t="s">
         <v>104</v>
       </c>
-      <c r="C10" s="40" t="s">
+      <c r="C10" s="32" t="s">
         <v>104</v>
       </c>
-      <c r="D10" s="40" t="s">
+      <c r="D10" s="32" t="s">
         <v>104</v>
       </c>
-      <c r="E10" s="55" t="s">
+      <c r="E10" s="41" t="s">
         <v>104</v>
       </c>
-      <c r="F10" s="40" t="s">
+      <c r="F10" s="32" t="s">
         <v>116</v>
       </c>
     </row>
@@ -9861,98 +10070,98 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="33" t="s">
         <v>120</v>
       </c>
-      <c r="B1" s="42" t="s">
+      <c r="B1" s="34" t="s">
         <v>121</v>
       </c>
-      <c r="C1" s="42" t="s">
+      <c r="C1" s="34" t="s">
         <v>122</v>
       </c>
-      <c r="D1" s="42" t="s">
+      <c r="D1" s="34" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="59" t="s">
         <v>92</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="35" t="s">
         <v>124</v>
       </c>
-      <c r="C2" s="45" t="s">
+      <c r="C2" s="62" t="s">
         <v>125</v>
       </c>
-      <c r="D2" s="43" t="s">
+      <c r="D2" s="59" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="46"/>
-      <c r="B3" s="44" t="s">
+      <c r="A3" s="60"/>
+      <c r="B3" s="35" t="s">
         <v>127</v>
       </c>
-      <c r="C3" s="47"/>
-      <c r="D3" s="46"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="60"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="46"/>
-      <c r="B4" s="44" t="s">
+      <c r="A4" s="60"/>
+      <c r="B4" s="35" t="s">
         <v>128</v>
       </c>
-      <c r="C4" s="47"/>
-      <c r="D4" s="46"/>
+      <c r="C4" s="63"/>
+      <c r="D4" s="60"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="46"/>
-      <c r="B5" s="44" t="s">
+      <c r="A5" s="60"/>
+      <c r="B5" s="35" t="s">
         <v>129</v>
       </c>
-      <c r="C5" s="47"/>
-      <c r="D5" s="46"/>
+      <c r="C5" s="63"/>
+      <c r="D5" s="60"/>
     </row>
     <row r="6" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="48"/>
-      <c r="B6" s="44" t="s">
+      <c r="A6" s="61"/>
+      <c r="B6" s="35" t="s">
         <v>130</v>
       </c>
-      <c r="C6" s="49"/>
-      <c r="D6" s="48"/>
+      <c r="C6" s="64"/>
+      <c r="D6" s="61"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="43" t="s">
+      <c r="A7" s="59" t="s">
         <v>131</v>
       </c>
-      <c r="B7" s="50" t="s">
+      <c r="B7" s="38" t="s">
         <v>132</v>
       </c>
-      <c r="C7" s="45" t="s">
+      <c r="C7" s="62" t="s">
         <v>133</v>
       </c>
-      <c r="D7" s="43" t="s">
+      <c r="D7" s="59" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="48"/>
-      <c r="B8" s="51" t="s">
+      <c r="A8" s="61"/>
+      <c r="B8" s="39" t="s">
         <v>135</v>
       </c>
-      <c r="C8" s="49"/>
-      <c r="D8" s="48"/>
+      <c r="C8" s="64"/>
+      <c r="D8" s="61"/>
     </row>
     <row r="9" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="52" t="s">
+      <c r="A9" s="36" t="s">
         <v>136</v>
       </c>
-      <c r="B9" s="51" t="s">
+      <c r="B9" s="39" t="s">
         <v>137</v>
       </c>
-      <c r="C9" s="53" t="s">
+      <c r="C9" s="37" t="s">
         <v>138</v>
       </c>
-      <c r="D9" s="54" t="s">
+      <c r="D9" s="40" t="s">
         <v>139</v>
       </c>
     </row>
@@ -9979,58 +10188,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="44" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="62" t="s">
+      <c r="B1" s="45" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="31" t="s">
         <v>141</v>
       </c>
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="41" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="32" t="s">
         <v>143</v>
       </c>
-      <c r="B3" s="55" t="s">
+      <c r="B3" s="41" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="39" t="s">
+      <c r="A4" s="31" t="s">
         <v>145</v>
       </c>
-      <c r="B4" s="55" t="s">
+      <c r="B4" s="41" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="39" t="s">
+      <c r="A5" s="31" t="s">
         <v>147</v>
       </c>
-      <c r="B5" s="55" t="s">
+      <c r="B5" s="41" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="39" t="s">
+      <c r="A6" s="31" t="s">
         <v>149</v>
       </c>
-      <c r="B6" s="55" t="s">
+      <c r="B6" s="41" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="39" t="s">
+      <c r="A7" s="31" t="s">
         <v>151</v>
       </c>
-      <c r="B7" s="55" t="s">
+      <c r="B7" s="41" t="s">
         <v>152</v>
       </c>
     </row>
@@ -10052,154 +10261,154 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="46" t="s">
         <v>210</v>
       </c>
-      <c r="B1" s="63" t="s">
+      <c r="B1" s="46" t="s">
         <v>153</v>
       </c>
-      <c r="C1" s="64" t="s">
+      <c r="C1" s="47" t="s">
         <v>154</v>
       </c>
-      <c r="D1" s="70" t="s">
+      <c r="D1" s="53" t="s">
         <v>155</v>
       </c>
-      <c r="E1" s="64" t="s">
+      <c r="E1" s="47" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="32" t="s">
         <v>202</v>
       </c>
-      <c r="B2" s="40" t="s">
+      <c r="B2" s="32" t="s">
         <v>157</v>
       </c>
-      <c r="C2" s="55" t="s">
+      <c r="C2" s="41" t="s">
         <v>158</v>
       </c>
-      <c r="D2" s="71">
+      <c r="D2" s="54">
         <v>90</v>
       </c>
-      <c r="E2" s="55" t="s">
+      <c r="E2" s="41" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="32" t="s">
         <v>202</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="32" t="s">
         <v>159</v>
       </c>
-      <c r="C3" s="55" t="s">
+      <c r="C3" s="41" t="s">
         <v>160</v>
       </c>
-      <c r="D3" s="71">
+      <c r="D3" s="54">
         <v>75</v>
       </c>
-      <c r="E3" s="55" t="s">
+      <c r="E3" s="41" t="s">
         <v>221</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="32" t="s">
         <v>202</v>
       </c>
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="32" t="s">
         <v>203</v>
       </c>
-      <c r="C4" s="55" t="s">
+      <c r="C4" s="41" t="s">
         <v>161</v>
       </c>
-      <c r="D4" s="72">
+      <c r="D4" s="55">
         <v>60</v>
       </c>
-      <c r="E4" s="55" t="s">
+      <c r="E4" s="41" t="s">
         <v>219</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="40" t="s">
+      <c r="A5" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="40" t="s">
+      <c r="B5" s="32" t="s">
         <v>204</v>
       </c>
-      <c r="C5" s="55" t="s">
+      <c r="C5" s="41" t="s">
         <v>205</v>
       </c>
-      <c r="D5" s="71">
+      <c r="D5" s="54">
         <v>70</v>
       </c>
-      <c r="E5" s="55" t="s">
+      <c r="E5" s="41" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="40" t="s">
+      <c r="A6" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="B6" s="40" t="s">
+      <c r="B6" s="32" t="s">
         <v>209</v>
       </c>
-      <c r="C6" s="55" t="s">
+      <c r="C6" s="41" t="s">
         <v>207</v>
       </c>
-      <c r="D6" s="72">
+      <c r="D6" s="55">
         <v>55</v>
       </c>
-      <c r="E6" s="55" t="s">
+      <c r="E6" s="41" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="40" t="s">
+      <c r="A7" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="B7" s="40" t="s">
+      <c r="B7" s="32" t="s">
         <v>159</v>
       </c>
-      <c r="C7" s="55" t="s">
+      <c r="C7" s="41" t="s">
         <v>208</v>
       </c>
-      <c r="D7" s="73">
+      <c r="D7" s="56">
         <v>40</v>
       </c>
-      <c r="E7" s="55" t="s">
+      <c r="E7" s="41" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D8" s="74"/>
+      <c r="D8" s="57"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D11" s="67">
+      <c r="D11" s="50">
         <v>90</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D12" s="65">
+      <c r="D12" s="48">
         <v>75</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D13" s="68">
+      <c r="D13" s="51">
         <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D14" s="65">
+      <c r="D14" s="48">
         <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D15" s="66">
+      <c r="D15" s="49">
         <v>55</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D16" s="69">
+      <c r="D16" s="52">
         <v>40</v>
       </c>
     </row>
@@ -10221,104 +10430,104 @@
       </c>
     </row>
     <row r="20" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="75" t="s">
+      <c r="A20" s="58" t="s">
         <v>202</v>
       </c>
-      <c r="B20" s="75" t="s">
+      <c r="B20" s="58" t="s">
         <v>157</v>
       </c>
-      <c r="C20" s="75" t="s">
+      <c r="C20" s="58" t="s">
         <v>158</v>
       </c>
-      <c r="D20" s="75">
+      <c r="D20" s="58">
         <v>90</v>
       </c>
-      <c r="E20" s="75" t="s">
+      <c r="E20" s="58" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="75" t="s">
+      <c r="A21" s="58" t="s">
         <v>202</v>
       </c>
-      <c r="B21" s="75" t="s">
+      <c r="B21" s="58" t="s">
         <v>159</v>
       </c>
-      <c r="C21" s="75" t="s">
+      <c r="C21" s="58" t="s">
         <v>160</v>
       </c>
-      <c r="D21" s="75">
+      <c r="D21" s="58">
         <v>75</v>
       </c>
-      <c r="E21" s="75" t="s">
+      <c r="E21" s="58" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" s="75" t="s">
+      <c r="A22" s="58" t="s">
         <v>202</v>
       </c>
-      <c r="B22" s="75" t="s">
+      <c r="B22" s="58" t="s">
         <v>203</v>
       </c>
-      <c r="C22" s="75" t="s">
+      <c r="C22" s="58" t="s">
         <v>161</v>
       </c>
-      <c r="D22" s="75">
+      <c r="D22" s="58">
         <v>60</v>
       </c>
-      <c r="E22" s="75" t="s">
+      <c r="E22" s="58" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="75" t="s">
+      <c r="A23" s="58" t="s">
         <v>47</v>
       </c>
-      <c r="B23" s="75" t="s">
+      <c r="B23" s="58" t="s">
         <v>204</v>
       </c>
-      <c r="C23" s="75" t="s">
+      <c r="C23" s="58" t="s">
         <v>205</v>
       </c>
-      <c r="D23" s="75">
+      <c r="D23" s="58">
         <v>70</v>
       </c>
-      <c r="E23" s="75" t="s">
+      <c r="E23" s="58" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="75" t="s">
+      <c r="A24" s="58" t="s">
         <v>47</v>
       </c>
-      <c r="B24" s="75" t="s">
+      <c r="B24" s="58" t="s">
         <v>209</v>
       </c>
-      <c r="C24" s="75" t="s">
+      <c r="C24" s="58" t="s">
         <v>207</v>
       </c>
-      <c r="D24" s="75">
+      <c r="D24" s="58">
         <v>55</v>
       </c>
-      <c r="E24" s="75" t="s">
+      <c r="E24" s="58" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="75" t="s">
+      <c r="A25" s="58" t="s">
         <v>47</v>
       </c>
-      <c r="B25" s="75" t="s">
+      <c r="B25" s="58" t="s">
         <v>159</v>
       </c>
-      <c r="C25" s="75" t="s">
+      <c r="C25" s="58" t="s">
         <v>208</v>
       </c>
-      <c r="D25" s="75">
+      <c r="D25" s="58">
         <v>40</v>
       </c>
-      <c r="E25" s="75" t="s">
+      <c r="E25" s="58" t="s">
         <v>216</v>
       </c>
     </row>
@@ -10332,138 +10541,137 @@
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="20.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" style="38" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.5703125" style="38" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.5703125" style="38" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29" style="38" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="38"/>
+    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="33" t="s">
         <v>162</v>
       </c>
-      <c r="B1" s="42" t="s">
+      <c r="B1" s="34" t="s">
         <v>163</v>
       </c>
-      <c r="C1" s="42" t="s">
+      <c r="C1" s="34" t="s">
         <v>164</v>
       </c>
-      <c r="D1" s="42" t="s">
+      <c r="D1" s="34" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="65" t="s">
         <v>166</v>
       </c>
-      <c r="B2" s="56" t="s">
+      <c r="B2" s="42" t="s">
         <v>167</v>
       </c>
-      <c r="C2" s="56" t="s">
+      <c r="C2" s="42" t="s">
         <v>168</v>
       </c>
-      <c r="D2" s="56" t="s">
+      <c r="D2" s="42" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="58"/>
-      <c r="B3" s="56" t="s">
+      <c r="A3" s="66"/>
+      <c r="B3" s="42" t="s">
         <v>170</v>
       </c>
-      <c r="C3" s="56" t="s">
+      <c r="C3" s="42" t="s">
         <v>171</v>
       </c>
-      <c r="D3" s="56" t="s">
+      <c r="D3" s="42" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="58"/>
-      <c r="B4" s="56" t="s">
+      <c r="A4" s="66"/>
+      <c r="B4" s="42" t="s">
         <v>173</v>
       </c>
-      <c r="C4" s="56" t="s">
+      <c r="C4" s="42" t="s">
         <v>174</v>
       </c>
-      <c r="D4" s="56" t="s">
+      <c r="D4" s="42" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="59"/>
-      <c r="B5" s="56" t="s">
+      <c r="A5" s="67"/>
+      <c r="B5" s="42" t="s">
         <v>176</v>
       </c>
-      <c r="C5" s="56" t="s">
+      <c r="C5" s="42" t="s">
         <v>177</v>
       </c>
-      <c r="D5" s="56" t="s">
+      <c r="D5" s="42" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="6" spans="1:4" s="60" customFormat="1" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="57" t="s">
+    <row r="6" spans="1:4" s="43" customFormat="1" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="65" t="s">
         <v>179</v>
       </c>
-      <c r="B6" s="56" t="s">
+      <c r="B6" s="42" t="s">
         <v>180</v>
       </c>
-      <c r="C6" s="56" t="s">
+      <c r="C6" s="42" t="s">
         <v>181</v>
       </c>
-      <c r="D6" s="56" t="s">
+      <c r="D6" s="42" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="7" spans="1:4" s="60" customFormat="1" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="58"/>
-      <c r="B7" s="56" t="s">
+    <row r="7" spans="1:4" s="43" customFormat="1" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="66"/>
+      <c r="B7" s="42" t="s">
         <v>183</v>
       </c>
-      <c r="C7" s="56" t="s">
+      <c r="C7" s="42" t="s">
         <v>184</v>
       </c>
-      <c r="D7" s="56" t="s">
+      <c r="D7" s="42" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="8" spans="1:4" s="60" customFormat="1" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="59"/>
-      <c r="B8" s="56" t="s">
+    <row r="8" spans="1:4" s="43" customFormat="1" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="67"/>
+      <c r="B8" s="42" t="s">
         <v>186</v>
       </c>
-      <c r="C8" s="56" t="s">
+      <c r="C8" s="42" t="s">
         <v>187</v>
       </c>
-      <c r="D8" s="56" t="s">
+      <c r="D8" s="42" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="9" spans="1:4" s="60" customFormat="1" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="57" t="s">
+    <row r="9" spans="1:4" s="43" customFormat="1" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="65" t="s">
         <v>189</v>
       </c>
-      <c r="B9" s="56" t="s">
+      <c r="B9" s="42" t="s">
         <v>190</v>
       </c>
-      <c r="C9" s="56" t="s">
+      <c r="C9" s="42" t="s">
         <v>191</v>
       </c>
-      <c r="D9" s="56" t="s">
+      <c r="D9" s="42" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="10" spans="1:4" s="60" customFormat="1" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="59"/>
-      <c r="B10" s="56" t="s">
+    <row r="10" spans="1:4" s="43" customFormat="1" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="67"/>
+      <c r="B10" s="42" t="s">
         <v>193</v>
       </c>
-      <c r="C10" s="56" t="s">
+      <c r="C10" s="42" t="s">
         <v>194</v>
       </c>
-      <c r="D10" s="56" t="s">
+      <c r="D10" s="42" t="s">
         <v>195</v>
       </c>
     </row>
@@ -10478,6 +10686,277 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40F016E6-E3BE-4013-A30D-53A57E6A2B2E}">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.42578125" style="43" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" style="43" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.28515625" style="43" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" style="43" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" style="43" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" style="43" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8" style="43" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="43"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="72" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="73" t="s">
+        <v>250</v>
+      </c>
+      <c r="C1" s="74" t="s">
+        <v>251</v>
+      </c>
+      <c r="D1" s="74" t="s">
+        <v>252</v>
+      </c>
+      <c r="E1" s="73" t="s">
+        <v>253</v>
+      </c>
+      <c r="F1" s="74" t="s">
+        <v>254</v>
+      </c>
+      <c r="G1" s="74" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="37" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="75">
+        <v>31.637035000000001</v>
+      </c>
+      <c r="C2" s="76">
+        <v>0.35705003000000002</v>
+      </c>
+      <c r="D2" s="76">
+        <v>0.32810002999999999</v>
+      </c>
+      <c r="E2" s="77">
+        <v>0.18</v>
+      </c>
+      <c r="F2" s="78">
+        <v>16.132999999999999</v>
+      </c>
+      <c r="G2" s="79">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="37" t="s">
+        <v>241</v>
+      </c>
+      <c r="B3" s="75">
+        <v>6.5364636999999997</v>
+      </c>
+      <c r="C3" s="76">
+        <v>0.28667998</v>
+      </c>
+      <c r="D3" s="76">
+        <v>9.1050000000000006E-2</v>
+      </c>
+      <c r="E3" s="77">
+        <v>-2.3E-2</v>
+      </c>
+      <c r="F3" s="78">
+        <v>482.32900000000001</v>
+      </c>
+      <c r="G3" s="79">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="37" t="s">
+        <v>242</v>
+      </c>
+      <c r="B4" s="75">
+        <v>5.497217</v>
+      </c>
+      <c r="C4" s="76">
+        <v>0.21410000000000001</v>
+      </c>
+      <c r="D4" s="76">
+        <v>0.16166</v>
+      </c>
+      <c r="E4" s="77">
+        <v>1.2E-2</v>
+      </c>
+      <c r="F4" s="78">
+        <v>107.863</v>
+      </c>
+      <c r="G4" s="79">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="37" t="s">
+        <v>243</v>
+      </c>
+      <c r="B5" s="75">
+        <v>15.653903</v>
+      </c>
+      <c r="C5" s="76">
+        <v>0.12024</v>
+      </c>
+      <c r="D5" s="76">
+        <v>0.128</v>
+      </c>
+      <c r="E5" s="77">
+        <v>5.1999999999999998E-2</v>
+      </c>
+      <c r="F5" s="78">
+        <v>40.908999999999999</v>
+      </c>
+      <c r="G5" s="79">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="37" t="s">
+        <v>244</v>
+      </c>
+      <c r="B6" s="75">
+        <v>76.340819999999994</v>
+      </c>
+      <c r="C6" s="76">
+        <v>0.10027</v>
+      </c>
+      <c r="D6" s="76">
+        <v>9.307E-2</v>
+      </c>
+      <c r="E6" s="77">
+        <v>0.01</v>
+      </c>
+      <c r="F6" s="78">
+        <v>36.442999999999998</v>
+      </c>
+      <c r="G6" s="79">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="37" t="s">
+        <v>245</v>
+      </c>
+      <c r="B7" s="75">
+        <v>14.035971</v>
+      </c>
+      <c r="C7" s="76">
+        <v>0.16822999999999999</v>
+      </c>
+      <c r="D7" s="76">
+        <v>0.11407</v>
+      </c>
+      <c r="E7" s="77">
+        <v>0.02</v>
+      </c>
+      <c r="F7" s="78">
+        <v>67.388999999999996</v>
+      </c>
+      <c r="G7" s="79">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="37" t="s">
+        <v>246</v>
+      </c>
+      <c r="B8" s="75">
+        <v>15.604316000000001</v>
+      </c>
+      <c r="C8" s="76">
+        <v>0.16822999999999999</v>
+      </c>
+      <c r="D8" s="76">
+        <v>0.11407</v>
+      </c>
+      <c r="E8" s="77">
+        <v>0.02</v>
+      </c>
+      <c r="F8" s="78">
+        <v>67.388999999999996</v>
+      </c>
+      <c r="G8" s="79">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="37" t="s">
+        <v>247</v>
+      </c>
+      <c r="B9" s="75">
+        <v>31.338873</v>
+      </c>
+      <c r="C9" s="76">
+        <v>0.35705003000000002</v>
+      </c>
+      <c r="D9" s="76">
+        <v>0.32810002999999999</v>
+      </c>
+      <c r="E9" s="77">
+        <v>0.18</v>
+      </c>
+      <c r="F9" s="78">
+        <v>16.132999999999999</v>
+      </c>
+      <c r="G9" s="79">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="37" t="s">
+        <v>248</v>
+      </c>
+      <c r="B10" s="75"/>
+      <c r="C10" s="76">
+        <v>0.36701</v>
+      </c>
+      <c r="D10" s="76">
+        <v>1.968E-2</v>
+      </c>
+      <c r="E10" s="77">
+        <v>0.111</v>
+      </c>
+      <c r="F10" s="78">
+        <v>572.03200000000004</v>
+      </c>
+      <c r="G10" s="79">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="37" t="s">
+        <v>249</v>
+      </c>
+      <c r="B11" s="75">
+        <v>15.604316000000001</v>
+      </c>
+      <c r="C11" s="76">
+        <v>0.191165</v>
+      </c>
+      <c r="D11" s="76">
+        <v>0.11407</v>
+      </c>
+      <c r="E11" s="77">
+        <v>0.02</v>
+      </c>
+      <c r="F11" s="78">
+        <v>67.388999999999996</v>
+      </c>
+      <c r="G11" s="79">
+        <v>7.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37F48F30-B7F9-4DA6-91B4-4AA828DEC5EB}">
   <sheetPr>
     <tabColor rgb="FF92D050"/>
@@ -10489,7 +10968,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{573CE6C7-0819-4144-9C76-88AA858FAEA7}">
   <dimension ref="A1:J23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -11236,454 +11715,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{997BFE89-0423-4747-91F1-EB3B75F2F832}">
-  <dimension ref="A1:N10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F1" t="s">
-        <v>26</v>
-      </c>
-      <c r="G1" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" t="s">
-        <v>28</v>
-      </c>
-      <c r="I1" t="s">
-        <v>29</v>
-      </c>
-      <c r="J1" t="s">
-        <v>30</v>
-      </c>
-      <c r="K1" t="s">
-        <v>31</v>
-      </c>
-      <c r="L1" t="s">
-        <v>32</v>
-      </c>
-      <c r="M1" t="s">
-        <v>33</v>
-      </c>
-      <c r="N1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2">
-        <v>3</v>
-      </c>
-      <c r="C2">
-        <v>1.1539999999999999</v>
-      </c>
-      <c r="D2">
-        <v>100</v>
-      </c>
-      <c r="E2">
-        <v>1.226</v>
-      </c>
-      <c r="F2">
-        <v>100</v>
-      </c>
-      <c r="G2">
-        <v>9.0999999999999998E-2</v>
-      </c>
-      <c r="H2">
-        <v>66.67</v>
-      </c>
-      <c r="I2">
-        <v>-0.247</v>
-      </c>
-      <c r="J2">
-        <v>33.33</v>
-      </c>
-      <c r="K2">
-        <v>-1.7989999999999999</v>
-      </c>
-      <c r="L2">
-        <v>66.67</v>
-      </c>
-      <c r="M2">
-        <v>-6.0869999999999997</v>
-      </c>
-      <c r="N2">
-        <v>33.33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3">
-        <v>4</v>
-      </c>
-      <c r="C3">
-        <v>-0.57999999999999996</v>
-      </c>
-      <c r="D3">
-        <v>25</v>
-      </c>
-      <c r="E3">
-        <v>0.13300000000000001</v>
-      </c>
-      <c r="F3">
-        <v>25</v>
-      </c>
-      <c r="G3">
-        <v>-0.64500000000000002</v>
-      </c>
-      <c r="H3">
-        <v>25</v>
-      </c>
-      <c r="I3">
-        <v>-0.53900000000000003</v>
-      </c>
-      <c r="J3">
-        <v>25</v>
-      </c>
-      <c r="K3">
-        <v>1.611</v>
-      </c>
-      <c r="L3">
-        <v>25</v>
-      </c>
-      <c r="M3">
-        <v>15.06</v>
-      </c>
-      <c r="N3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4">
-        <v>3</v>
-      </c>
-      <c r="C4">
-        <v>-1.1359999999999999</v>
-      </c>
-      <c r="D4">
-        <v>33.33</v>
-      </c>
-      <c r="E4">
-        <v>-1.0109999999999999</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>-0.86299999999999999</v>
-      </c>
-      <c r="H4">
-        <v>33.33</v>
-      </c>
-      <c r="I4">
-        <v>-0.21299999999999999</v>
-      </c>
-      <c r="J4">
-        <v>66.67</v>
-      </c>
-      <c r="K4">
-        <v>2.76</v>
-      </c>
-      <c r="L4">
-        <v>66.67</v>
-      </c>
-      <c r="M4">
-        <v>7.1580000000000004</v>
-      </c>
-      <c r="N4">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>32.093000000000004</v>
-      </c>
-      <c r="D5">
-        <v>100</v>
-      </c>
-      <c r="E5">
-        <v>33.332999999999998</v>
-      </c>
-      <c r="F5">
-        <v>100</v>
-      </c>
-      <c r="G5">
-        <v>53.444000000000003</v>
-      </c>
-      <c r="H5">
-        <v>100</v>
-      </c>
-      <c r="I5">
-        <v>44.877000000000002</v>
-      </c>
-      <c r="J5">
-        <v>100</v>
-      </c>
-      <c r="K5">
-        <v>51.631</v>
-      </c>
-      <c r="L5">
-        <v>100</v>
-      </c>
-      <c r="M5">
-        <v>63.975999999999999</v>
-      </c>
-      <c r="N5">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6">
-        <v>3</v>
-      </c>
-      <c r="C6">
-        <v>5.3710000000000004</v>
-      </c>
-      <c r="D6">
-        <v>100</v>
-      </c>
-      <c r="E6">
-        <v>3.0259999999999998</v>
-      </c>
-      <c r="F6">
-        <v>100</v>
-      </c>
-      <c r="G6">
-        <v>5.2670000000000003</v>
-      </c>
-      <c r="H6">
-        <v>100</v>
-      </c>
-      <c r="I6">
-        <v>7.0709999999999997</v>
-      </c>
-      <c r="J6">
-        <v>100</v>
-      </c>
-      <c r="K6">
-        <v>12.648999999999999</v>
-      </c>
-      <c r="L6">
-        <v>100</v>
-      </c>
-      <c r="M6">
-        <v>5.1559999999999997</v>
-      </c>
-      <c r="N6">
-        <v>66.67</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7">
-        <v>5</v>
-      </c>
-      <c r="C7">
-        <v>1.1679999999999999</v>
-      </c>
-      <c r="D7">
-        <v>40</v>
-      </c>
-      <c r="E7">
-        <v>0.81</v>
-      </c>
-      <c r="F7">
-        <v>60</v>
-      </c>
-      <c r="G7">
-        <v>0.186</v>
-      </c>
-      <c r="H7">
-        <v>60</v>
-      </c>
-      <c r="I7">
-        <v>-1.1160000000000001</v>
-      </c>
-      <c r="J7">
-        <v>40</v>
-      </c>
-      <c r="K7">
-        <v>-2.5070000000000001</v>
-      </c>
-      <c r="L7">
-        <v>20</v>
-      </c>
-      <c r="M7">
-        <v>-2.4409999999999998</v>
-      </c>
-      <c r="N7">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8">
-        <v>1</v>
-      </c>
-      <c r="C8">
-        <v>1.288</v>
-      </c>
-      <c r="D8">
-        <v>100</v>
-      </c>
-      <c r="E8">
-        <v>0.86</v>
-      </c>
-      <c r="F8">
-        <v>100</v>
-      </c>
-      <c r="G8">
-        <v>1.661</v>
-      </c>
-      <c r="H8">
-        <v>100</v>
-      </c>
-      <c r="I8">
-        <v>2.7719999999999998</v>
-      </c>
-      <c r="J8">
-        <v>100</v>
-      </c>
-      <c r="K8">
-        <v>17.22</v>
-      </c>
-      <c r="L8">
-        <v>100</v>
-      </c>
-      <c r="M8">
-        <v>19.041</v>
-      </c>
-      <c r="N8">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9">
-        <v>2</v>
-      </c>
-      <c r="C9">
-        <v>-1.0649999999999999</v>
-      </c>
-      <c r="D9">
-        <v>50</v>
-      </c>
-      <c r="E9">
-        <v>-3.97</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
-      <c r="G9">
-        <v>-4.1310000000000002</v>
-      </c>
-      <c r="H9">
-        <v>0</v>
-      </c>
-      <c r="I9">
-        <v>-2.4729999999999999</v>
-      </c>
-      <c r="J9">
-        <v>50</v>
-      </c>
-      <c r="K9">
-        <v>2.1720000000000002</v>
-      </c>
-      <c r="L9">
-        <v>50</v>
-      </c>
-      <c r="M9">
-        <v>-9.6709999999999994</v>
-      </c>
-      <c r="N9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10">
-        <v>22</v>
-      </c>
-      <c r="C10">
-        <v>2.3149999999999999</v>
-      </c>
-      <c r="D10">
-        <v>59.09</v>
-      </c>
-      <c r="E10">
-        <v>1.8440000000000001</v>
-      </c>
-      <c r="F10">
-        <v>54.55</v>
-      </c>
-      <c r="G10">
-        <v>2.6669999999999998</v>
-      </c>
-      <c r="H10">
-        <v>54.55</v>
-      </c>
-      <c r="I10">
-        <v>2.4910000000000001</v>
-      </c>
-      <c r="J10">
-        <v>54.55</v>
-      </c>
-      <c r="K10">
-        <v>4.9059999999999997</v>
-      </c>
-      <c r="L10">
-        <v>54.55</v>
-      </c>
-      <c r="M10">
-        <v>5.9269999999999996</v>
-      </c>
-      <c r="N10">
-        <v>63.64</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>